<commit_message>
Oferta: podgląd przed pobraniem Worda, logo bez fetch, H1/H2 bez pogrubionej cyfry
Opcja 2500 kg domyślnie wyłączona; zmiana zysku nie zwija sekcji formularza.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XygCrjT9K7zVw2zg8hs3qQ
</commit_message>
<xml_diff>
--- a/kalkulator-nk38/przyklady/Kalkulator_ul_Brzozowa_9_Poznan_NK38.xlsx
+++ b/kalkulator-nk38/przyklady/Kalkulator_ul_Brzozowa_9_Poznan_NK38.xlsx
@@ -168,10 +168,10 @@
     <t>ul. Brzozowa 9, Poznań</t>
   </si>
   <si>
-    <t>21.10.2026, 17:30</t>
-  </si>
-  <si>
-    <t>Wygenerowano 27.10.2026, 17:30:55 · ceny netto w zł · szablon NK38</t>
+    <t>21.10.2026, 10:10</t>
+  </si>
+  <si>
+    <t>Wygenerowano 30.10.2026, 10:10:16 · ceny netto w zł · szablon NK38</t>
   </si>
   <si>
     <t>Cena</t>

</xml_diff>

<commit_message>
Opis wariantu: ręczna zmiana fragmentu nie wyłącza automatyki reszty; nagłówki oferty z następnym akapitem
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XygCrjT9K7zVw2zg8hs3qQ
</commit_message>
<xml_diff>
--- a/kalkulator-nk38/przyklady/Kalkulator_ul_Brzozowa_9_Poznan_NK38.xlsx
+++ b/kalkulator-nk38/przyklady/Kalkulator_ul_Brzozowa_9_Poznan_NK38.xlsx
@@ -22,10 +22,10 @@
     <t>ul. Brzozowa 9, Poznań</t>
   </si>
   <si>
-    <t>21.10.2026, 10:28</t>
-  </si>
-  <si>
-    <t>Wygenerowano 30.10.2026, 10:28:00 · ceny netto w zł · szablon NK38</t>
+    <t>21.10.2026, 11:44</t>
+  </si>
+  <si>
+    <t>Wygenerowano 30.10.2026, 11:44:46 · ceny netto w zł · szablon NK38</t>
   </si>
   <si>
     <t>Cena</t>
@@ -945,7 +945,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="bottom"/>
@@ -1130,8 +1130,11 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment indent="1"/>
     </xf>
+    <xf numFmtId="171" fontId="17" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" indent="3"/>
+    </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+      <alignment horizontal="right" indent="3"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2971,7 +2974,7 @@
       <c r="A122" s="63" t="s">
         <v>182</v>
       </c>
-      <c r="B122" s="62">
+      <c r="B122" s="64">
         <v>130</v>
       </c>
       <c r="C122" s="61" t="s">
@@ -2987,7 +2990,7 @@
       <c r="A123" s="63" t="s">
         <v>184</v>
       </c>
-      <c r="B123" s="62">
+      <c r="B123" s="64">
         <v>45</v>
       </c>
       <c r="C123" s="61" t="s">
@@ -3019,7 +3022,7 @@
       <c r="A125" s="63" t="s">
         <v>188</v>
       </c>
-      <c r="B125" s="64" t="s">
+      <c r="B125" s="65" t="s">
         <v>189</v>
       </c>
       <c r="C125" s="61" t="s">
@@ -3035,7 +3038,7 @@
       <c r="A126" s="63" t="s">
         <v>191</v>
       </c>
-      <c r="B126" s="64" t="s">
+      <c r="B126" s="65" t="s">
         <v>192</v>
       </c>
       <c r="C126" s="61" t="s">
@@ -3051,7 +3054,7 @@
       <c r="A127" s="63" t="s">
         <v>194</v>
       </c>
-      <c r="B127" s="64" t="s">
+      <c r="B127" s="65" t="s">
         <v>195</v>
       </c>
       <c r="C127" s="61" t="s">
@@ -3083,7 +3086,7 @@
       <c r="A129" s="63" t="s">
         <v>199</v>
       </c>
-      <c r="B129" s="62">
+      <c r="B129" s="64">
         <v>0</v>
       </c>
       <c r="C129" s="61" t="s">
@@ -3099,7 +3102,7 @@
       <c r="A130" s="63" t="s">
         <v>201</v>
       </c>
-      <c r="B130" s="62">
+      <c r="B130" s="64">
         <v>500</v>
       </c>
       <c r="C130" s="61" t="s">
@@ -3115,7 +3118,7 @@
       <c r="A131" s="63" t="s">
         <v>203</v>
       </c>
-      <c r="B131" s="62">
+      <c r="B131" s="64">
         <v>550</v>
       </c>
       <c r="C131" s="61" t="s">
@@ -3131,7 +3134,7 @@
       <c r="A132" s="63" t="s">
         <v>205</v>
       </c>
-      <c r="B132" s="62">
+      <c r="B132" s="64">
         <v>600</v>
       </c>
       <c r="C132" s="61" t="s">
@@ -3147,7 +3150,7 @@
       <c r="A133" s="63" t="s">
         <v>207</v>
       </c>
-      <c r="B133" s="62">
+      <c r="B133" s="64">
         <v>650</v>
       </c>
       <c r="C133" s="61" t="s">
@@ -3163,7 +3166,7 @@
       <c r="A134" s="63" t="s">
         <v>209</v>
       </c>
-      <c r="B134" s="62">
+      <c r="B134" s="64">
         <v>700</v>
       </c>
       <c r="C134" s="61" t="s">
@@ -3179,7 +3182,7 @@
       <c r="A135" s="63" t="s">
         <v>211</v>
       </c>
-      <c r="B135" s="62">
+      <c r="B135" s="64">
         <v>750</v>
       </c>
       <c r="C135" s="61" t="s">
@@ -3195,7 +3198,7 @@
       <c r="A136" s="63" t="s">
         <v>213</v>
       </c>
-      <c r="B136" s="62">
+      <c r="B136" s="64">
         <v>800</v>
       </c>
       <c r="C136" s="61" t="s">
@@ -3211,7 +3214,7 @@
       <c r="A137" s="63" t="s">
         <v>215</v>
       </c>
-      <c r="B137" s="62">
+      <c r="B137" s="64">
         <v>850</v>
       </c>
       <c r="C137" s="61" t="s">
@@ -3243,7 +3246,7 @@
       <c r="A139" s="63" t="s">
         <v>219</v>
       </c>
-      <c r="B139" s="62">
+      <c r="B139" s="64">
         <v>1170</v>
       </c>
       <c r="C139" s="61" t="s">
@@ -3259,7 +3262,7 @@
       <c r="A140" s="63" t="s">
         <v>221</v>
       </c>
-      <c r="B140" s="62">
+      <c r="B140" s="64">
         <v>1560</v>
       </c>
       <c r="C140" s="61" t="s">
@@ -3275,7 +3278,7 @@
       <c r="A141" s="63" t="s">
         <v>223</v>
       </c>
-      <c r="B141" s="62">
+      <c r="B141" s="64">
         <v>1820</v>
       </c>
       <c r="C141" s="61" t="s">
@@ -3291,7 +3294,7 @@
       <c r="A142" s="63" t="s">
         <v>225</v>
       </c>
-      <c r="B142" s="62">
+      <c r="B142" s="64">
         <v>3110</v>
       </c>
       <c r="C142" s="61" t="s">
@@ -3307,7 +3310,7 @@
       <c r="A143" s="63" t="s">
         <v>227</v>
       </c>
-      <c r="B143" s="62">
+      <c r="B143" s="64">
         <v>2340</v>
       </c>
       <c r="C143" s="61" t="s">
@@ -3323,7 +3326,7 @@
       <c r="A144" s="63" t="s">
         <v>229</v>
       </c>
-      <c r="B144" s="62">
+      <c r="B144" s="64">
         <v>10</v>
       </c>
       <c r="C144" s="61" t="s">
@@ -3339,7 +3342,7 @@
       <c r="A145" s="63" t="s">
         <v>231</v>
       </c>
-      <c r="B145" s="62">
+      <c r="B145" s="64">
         <v>20</v>
       </c>
       <c r="C145" s="61" t="s">
@@ -3371,7 +3374,7 @@
       <c r="A147" s="63" t="s">
         <v>235</v>
       </c>
-      <c r="B147" s="62">
+      <c r="B147" s="64">
         <v>45</v>
       </c>
       <c r="C147" t="s">

</xml_diff>

<commit_message>
Oferta: odmiana nazwy inwestycji we wstępie (ulica, miasto)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XygCrjT9K7zVw2zg8hs3qQ
</commit_message>
<xml_diff>
--- a/kalkulator-nk38/przyklady/Kalkulator_ul_Brzozowa_9_Poznan_NK38.xlsx
+++ b/kalkulator-nk38/przyklady/Kalkulator_ul_Brzozowa_9_Poznan_NK38.xlsx
@@ -22,10 +22,10 @@
     <t>ul. Brzozowa 9, Poznań</t>
   </si>
   <si>
-    <t>21.10.2026, 11:44</t>
-  </si>
-  <si>
-    <t>Wygenerowano 30.10.2026, 11:44:46 · ceny netto w zł · szablon NK38</t>
+    <t>21.10.2026, 12:42</t>
+  </si>
+  <si>
+    <t>Wygenerowano 30.10.2026, 12:42:34 · ceny netto w zł · szablon NK38</t>
   </si>
   <si>
     <t>Cena</t>

</xml_diff>